<commit_message>
no se la real
creo que actualice la matriz
</commit_message>
<xml_diff>
--- a/Actualizada_Matriz_Lf_Carpinter.xlsx
+++ b/Actualizada_Matriz_Lf_Carpinter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alejandra\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emmagammer\Downloads\taller_matrices\LF_carpenter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA742D6-6C15-4D7A-8DCB-972BF04D6931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DD6913-8E42-471C-9751-FF9D5D0DEFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" RF" sheetId="1" r:id="rId1"/>
@@ -1310,9 +1310,6 @@
     <t>Casos de Uso (A)</t>
   </si>
   <si>
-    <t>Cls_Pedido</t>
-  </si>
-  <si>
     <t>Pruebas</t>
   </si>
   <si>
@@ -1398,6 +1395,9 @@
   </si>
   <si>
     <t>a</t>
+  </si>
+  <si>
+    <t>SolicitudProyecto</t>
   </si>
 </sst>
 </file>
@@ -2361,6 +2361,26 @@
     <xf numFmtId="0" fontId="21" fillId="30" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="24" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2372,19 +2392,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2404,58 +2411,53 @@
     <xf numFmtId="0" fontId="19" fillId="21" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2467,18 +2469,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2761,16 +2761,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="117" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
     </row>
     <row r="2" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="40" t="s">
@@ -2856,20 +2856,20 @@
       <c r="B5" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="133" t="s">
+      <c r="C5" s="123" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="134"/>
-      <c r="E5" s="133" t="s">
+      <c r="D5" s="124"/>
+      <c r="E5" s="123" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="134"/>
-      <c r="G5" s="133" t="s">
+      <c r="F5" s="124"/>
+      <c r="G5" s="123" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="134"/>
-      <c r="I5" s="120"/>
-      <c r="J5" s="121"/>
+      <c r="H5" s="124"/>
+      <c r="I5" s="128"/>
+      <c r="J5" s="118"/>
       <c r="K5" s="10"/>
       <c r="L5" s="10"/>
       <c r="M5" s="10"/>
@@ -2890,7 +2890,7 @@
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="39" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B6" s="39" t="s">
         <v>12</v>
@@ -2934,10 +2934,10 @@
       <c r="AA6" s="12"/>
     </row>
     <row r="7" spans="1:27" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="122" t="s">
+      <c r="A7" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="122" t="s">
+      <c r="B7" s="119" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="49" t="s">
@@ -2971,8 +2971,8 @@
       <c r="S7" s="12"/>
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="123"/>
-      <c r="B8" s="123"/>
+      <c r="A8" s="120"/>
+      <c r="B8" s="120"/>
       <c r="C8" s="53" t="s">
         <v>27</v>
       </c>
@@ -3004,8 +3004,8 @@
       <c r="S8" s="12"/>
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="122"/>
-      <c r="B9" s="122"/>
+      <c r="A9" s="119"/>
+      <c r="B9" s="119"/>
       <c r="C9" s="49" t="s">
         <v>33</v>
       </c>
@@ -3037,8 +3037,8 @@
       <c r="S9" s="12"/>
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="123"/>
-      <c r="B10" s="123" t="s">
+      <c r="A10" s="120"/>
+      <c r="B10" s="120" t="s">
         <v>39</v>
       </c>
       <c r="C10" s="53" t="s">
@@ -3072,8 +3072,8 @@
       <c r="S10" s="12"/>
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="122"/>
-      <c r="B11" s="122"/>
+      <c r="A11" s="119"/>
+      <c r="B11" s="119"/>
       <c r="C11" s="49" t="s">
         <v>46</v>
       </c>
@@ -3105,7 +3105,7 @@
       <c r="S11" s="12"/>
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="123"/>
+      <c r="A12" s="120"/>
       <c r="B12" s="52" t="s">
         <v>52</v>
       </c>
@@ -3140,7 +3140,7 @@
       <c r="S12" s="12"/>
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="122"/>
+      <c r="A13" s="119"/>
       <c r="B13" s="48" t="s">
         <v>59</v>
       </c>
@@ -3175,8 +3175,8 @@
       <c r="S13" s="12"/>
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="123"/>
-      <c r="B14" s="123" t="s">
+      <c r="A14" s="120"/>
+      <c r="B14" s="120" t="s">
         <v>66</v>
       </c>
       <c r="C14" s="53" t="s">
@@ -3210,8 +3210,8 @@
       <c r="S14" s="12"/>
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="122"/>
-      <c r="B15" s="122"/>
+      <c r="A15" s="119"/>
+      <c r="B15" s="119"/>
       <c r="C15" s="49" t="s">
         <v>73</v>
       </c>
@@ -3243,8 +3243,8 @@
       <c r="S15" s="12"/>
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="123"/>
-      <c r="B16" s="123"/>
+      <c r="A16" s="120"/>
+      <c r="B16" s="120"/>
       <c r="C16" s="53" t="s">
         <v>79</v>
       </c>
@@ -3276,10 +3276,10 @@
       <c r="S16" s="12"/>
     </row>
     <row r="17" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="125" t="s">
+      <c r="A17" s="121" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="125" t="s">
+      <c r="B17" s="121" t="s">
         <v>86</v>
       </c>
       <c r="C17" s="57" t="s">
@@ -3313,8 +3313,8 @@
       <c r="S17" s="12"/>
     </row>
     <row r="18" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="124"/>
-      <c r="B18" s="124"/>
+      <c r="A18" s="122"/>
+      <c r="B18" s="122"/>
       <c r="C18" s="60" t="s">
         <v>93</v>
       </c>
@@ -3346,7 +3346,7 @@
       <c r="S18" s="12"/>
     </row>
     <row r="19" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="125"/>
+      <c r="A19" s="121"/>
       <c r="B19" s="56" t="s">
         <v>99</v>
       </c>
@@ -3381,8 +3381,8 @@
       <c r="S19" s="12"/>
     </row>
     <row r="20" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="124"/>
-      <c r="B20" s="124" t="s">
+      <c r="A20" s="122"/>
+      <c r="B20" s="122" t="s">
         <v>106</v>
       </c>
       <c r="C20" s="60" t="s">
@@ -3416,8 +3416,8 @@
       <c r="S20" s="12"/>
     </row>
     <row r="21" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="125"/>
-      <c r="B21" s="125"/>
+      <c r="A21" s="121"/>
+      <c r="B21" s="121"/>
       <c r="C21" s="57" t="s">
         <v>113</v>
       </c>
@@ -3449,8 +3449,8 @@
       <c r="S21" s="12"/>
     </row>
     <row r="22" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="124"/>
-      <c r="B22" s="124"/>
+      <c r="A22" s="122"/>
+      <c r="B22" s="122"/>
       <c r="C22" s="60" t="s">
         <v>119</v>
       </c>
@@ -3482,8 +3482,8 @@
       <c r="S22" s="12"/>
     </row>
     <row r="23" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="125"/>
-      <c r="B23" s="125"/>
+      <c r="A23" s="121"/>
+      <c r="B23" s="121"/>
       <c r="C23" s="57" t="s">
         <v>125</v>
       </c>
@@ -3515,8 +3515,8 @@
       <c r="S23" s="12"/>
     </row>
     <row r="24" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="124"/>
-      <c r="B24" s="124"/>
+      <c r="A24" s="122"/>
+      <c r="B24" s="122"/>
       <c r="C24" s="60" t="s">
         <v>131</v>
       </c>
@@ -3548,8 +3548,8 @@
       <c r="S24" s="12"/>
     </row>
     <row r="25" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="125"/>
-      <c r="B25" s="125"/>
+      <c r="A25" s="121"/>
+      <c r="B25" s="121"/>
       <c r="C25" s="57" t="s">
         <v>137</v>
       </c>
@@ -3581,8 +3581,8 @@
       <c r="S25" s="12"/>
     </row>
     <row r="26" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="124"/>
-      <c r="B26" s="124" t="s">
+      <c r="A26" s="122"/>
+      <c r="B26" s="122" t="s">
         <v>143</v>
       </c>
       <c r="C26" s="60" t="s">
@@ -3616,8 +3616,8 @@
       <c r="S26" s="12"/>
     </row>
     <row r="27" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="125"/>
-      <c r="B27" s="125"/>
+      <c r="A27" s="121"/>
+      <c r="B27" s="121"/>
       <c r="C27" s="57" t="s">
         <v>150</v>
       </c>
@@ -3649,7 +3649,7 @@
       <c r="S27" s="12"/>
     </row>
     <row r="28" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="126" t="s">
+      <c r="A28" s="129" t="s">
         <v>156</v>
       </c>
       <c r="B28" s="64" t="s">
@@ -3686,8 +3686,8 @@
       <c r="S28" s="12"/>
     </row>
     <row r="29" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="127"/>
-      <c r="B29" s="127" t="s">
+      <c r="A29" s="130"/>
+      <c r="B29" s="130" t="s">
         <v>164</v>
       </c>
       <c r="C29" s="68" t="s">
@@ -3721,8 +3721,8 @@
       <c r="S29" s="12"/>
     </row>
     <row r="30" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="126"/>
-      <c r="B30" s="126"/>
+      <c r="A30" s="129"/>
+      <c r="B30" s="129"/>
       <c r="C30" s="65" t="s">
         <v>171</v>
       </c>
@@ -3754,8 +3754,8 @@
       <c r="S30" s="12"/>
     </row>
     <row r="31" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="127"/>
-      <c r="B31" s="127" t="s">
+      <c r="A31" s="130"/>
+      <c r="B31" s="130" t="s">
         <v>177</v>
       </c>
       <c r="C31" s="68" t="s">
@@ -3789,8 +3789,8 @@
       <c r="S31" s="12"/>
     </row>
     <row r="32" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="126"/>
-      <c r="B32" s="126"/>
+      <c r="A32" s="129"/>
+      <c r="B32" s="129"/>
       <c r="C32" s="65" t="s">
         <v>184</v>
       </c>
@@ -3830,7 +3830,7 @@
       <c r="AA32" s="12"/>
     </row>
     <row r="33" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="130" t="s">
+      <c r="A33" s="133" t="s">
         <v>190</v>
       </c>
       <c r="B33" s="71" t="s">
@@ -3875,7 +3875,7 @@
       <c r="AA33" s="12"/>
     </row>
     <row r="34" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="131"/>
+      <c r="A34" s="134"/>
       <c r="B34" s="75" t="s">
         <v>198</v>
       </c>
@@ -3918,7 +3918,7 @@
       <c r="AA34" s="12"/>
     </row>
     <row r="35" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="130"/>
+      <c r="A35" s="133"/>
       <c r="B35" s="71" t="s">
         <v>205</v>
       </c>
@@ -3961,7 +3961,7 @@
       <c r="AA35" s="12"/>
     </row>
     <row r="36" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="131"/>
+      <c r="A36" s="134"/>
       <c r="B36" s="75" t="s">
         <v>212</v>
       </c>
@@ -4004,7 +4004,7 @@
       <c r="AA36" s="12"/>
     </row>
     <row r="37" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="128" t="s">
+      <c r="A37" s="131" t="s">
         <v>219</v>
       </c>
       <c r="B37" s="79" t="s">
@@ -4049,7 +4049,7 @@
       <c r="AA37" s="12"/>
     </row>
     <row r="38" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="129"/>
+      <c r="A38" s="132"/>
       <c r="B38" s="83" t="s">
         <v>227</v>
       </c>
@@ -4092,7 +4092,7 @@
       <c r="AA38" s="4"/>
     </row>
     <row r="39" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="128"/>
+      <c r="A39" s="131"/>
       <c r="B39" s="79" t="s">
         <v>234</v>
       </c>
@@ -4135,7 +4135,7 @@
       <c r="AA39" s="4"/>
     </row>
     <row r="40" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="129"/>
+      <c r="A40" s="132"/>
       <c r="B40" s="83" t="s">
         <v>241</v>
       </c>
@@ -4178,7 +4178,7 @@
       <c r="AA40" s="4"/>
     </row>
     <row r="41" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="117" t="s">
+      <c r="A41" s="125" t="s">
         <v>248</v>
       </c>
       <c r="B41" s="89" t="s">
@@ -4223,7 +4223,7 @@
       <c r="AA41" s="4"/>
     </row>
     <row r="42" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="117"/>
+      <c r="A42" s="125"/>
       <c r="B42" s="93" t="s">
         <v>256</v>
       </c>
@@ -4266,7 +4266,7 @@
       <c r="AA42" s="4"/>
     </row>
     <row r="43" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="118" t="s">
+      <c r="A43" s="126" t="s">
         <v>156</v>
       </c>
       <c r="B43" s="97" t="s">
@@ -4311,7 +4311,7 @@
       <c r="AA43" s="4"/>
     </row>
     <row r="44" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="118"/>
+      <c r="A44" s="126"/>
       <c r="B44" s="101" t="s">
         <v>263</v>
       </c>
@@ -4354,7 +4354,7 @@
       <c r="AA44" s="4"/>
     </row>
     <row r="45" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="119" t="s">
+      <c r="A45" s="127" t="s">
         <v>190</v>
       </c>
       <c r="B45" s="105" t="s">
@@ -4399,7 +4399,7 @@
       <c r="AA45" s="4"/>
     </row>
     <row r="46" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="119"/>
+      <c r="A46" s="127"/>
       <c r="B46" s="109" t="s">
         <v>283</v>
       </c>
@@ -4442,7 +4442,7 @@
       <c r="AA46" s="4"/>
     </row>
     <row r="47" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="119"/>
+      <c r="A47" s="127"/>
       <c r="B47" s="105" t="s">
         <v>283</v>
       </c>
@@ -12375,14 +12375,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A7:A16"/>
-    <mergeCell ref="A17:A27"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="B14:B16"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="A43:A44"/>
     <mergeCell ref="A45:A47"/>
@@ -12396,6 +12388,14 @@
     <mergeCell ref="A33:A36"/>
     <mergeCell ref="B29:B30"/>
     <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A7:A16"/>
+    <mergeCell ref="A17:A27"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -12420,15 +12420,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="138" t="s">
+      <c r="A1" s="145" t="s">
         <v>303</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
@@ -12450,14 +12450,14 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="141" t="s">
+      <c r="A2" s="138" t="s">
         <v>304</v>
       </c>
-      <c r="B2" s="142"/>
-      <c r="C2" s="142"/>
-      <c r="D2" s="142"/>
-      <c r="E2" s="142"/>
-      <c r="F2" s="142"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
       <c r="G2" s="38"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -12483,12 +12483,12 @@
       <c r="A3" s="39" t="s">
         <v>305</v>
       </c>
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="141" t="s">
         <v>306</v>
       </c>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="145"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="143"/>
       <c r="F3" s="39" t="s">
         <v>307</v>
       </c>
@@ -12522,9 +12522,9 @@
       <c r="B4" s="135" t="s">
         <v>310</v>
       </c>
-      <c r="C4" s="137"/>
-      <c r="D4" s="137"/>
-      <c r="E4" s="137"/>
+      <c r="C4" s="136"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="136"/>
       <c r="F4" s="135" t="s">
         <v>311</v>
       </c>
@@ -12552,13 +12552,13 @@
       <c r="Z4" s="4"/>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="137"/>
-      <c r="B5" s="137"/>
-      <c r="C5" s="137"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="137"/>
-      <c r="G5" s="137"/>
+      <c r="A5" s="136"/>
+      <c r="B5" s="136"/>
+      <c r="C5" s="136"/>
+      <c r="D5" s="136"/>
+      <c r="E5" s="136"/>
+      <c r="F5" s="136"/>
+      <c r="G5" s="136"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -12580,13 +12580,13 @@
       <c r="Z5" s="4"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="137"/>
-      <c r="B6" s="137"/>
-      <c r="C6" s="137"/>
-      <c r="D6" s="137"/>
-      <c r="E6" s="137"/>
-      <c r="F6" s="137"/>
-      <c r="G6" s="137"/>
+      <c r="A6" s="136"/>
+      <c r="B6" s="136"/>
+      <c r="C6" s="136"/>
+      <c r="D6" s="136"/>
+      <c r="E6" s="136"/>
+      <c r="F6" s="136"/>
+      <c r="G6" s="136"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
@@ -12608,13 +12608,13 @@
       <c r="Z6" s="4"/>
     </row>
     <row r="7" spans="1:26" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="137"/>
-      <c r="B7" s="137"/>
-      <c r="C7" s="137"/>
-      <c r="D7" s="137"/>
-      <c r="E7" s="137"/>
-      <c r="F7" s="137"/>
-      <c r="G7" s="137"/>
+      <c r="A7" s="136"/>
+      <c r="B7" s="136"/>
+      <c r="C7" s="136"/>
+      <c r="D7" s="136"/>
+      <c r="E7" s="136"/>
+      <c r="F7" s="136"/>
+      <c r="G7" s="136"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -12639,12 +12639,12 @@
       <c r="A8" s="135" t="s">
         <v>313</v>
       </c>
-      <c r="B8" s="139" t="s">
+      <c r="B8" s="140" t="s">
         <v>314</v>
       </c>
-      <c r="C8" s="137"/>
-      <c r="D8" s="137"/>
-      <c r="E8" s="137"/>
+      <c r="C8" s="136"/>
+      <c r="D8" s="136"/>
+      <c r="E8" s="136"/>
       <c r="F8" s="135" t="s">
         <v>315</v>
       </c>
@@ -12672,13 +12672,13 @@
       <c r="Z8" s="4"/>
     </row>
     <row r="9" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="137"/>
-      <c r="B9" s="137"/>
-      <c r="C9" s="137"/>
-      <c r="D9" s="137"/>
-      <c r="E9" s="137"/>
-      <c r="F9" s="137"/>
-      <c r="G9" s="137"/>
+      <c r="A9" s="136"/>
+      <c r="B9" s="136"/>
+      <c r="C9" s="136"/>
+      <c r="D9" s="136"/>
+      <c r="E9" s="136"/>
+      <c r="F9" s="136"/>
+      <c r="G9" s="136"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -12700,13 +12700,13 @@
       <c r="Z9" s="4"/>
     </row>
     <row r="10" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="137"/>
-      <c r="B10" s="137"/>
-      <c r="C10" s="137"/>
-      <c r="D10" s="137"/>
-      <c r="E10" s="137"/>
-      <c r="F10" s="137"/>
-      <c r="G10" s="137"/>
+      <c r="A10" s="136"/>
+      <c r="B10" s="136"/>
+      <c r="C10" s="136"/>
+      <c r="D10" s="136"/>
+      <c r="E10" s="136"/>
+      <c r="F10" s="136"/>
+      <c r="G10" s="136"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -12728,13 +12728,13 @@
       <c r="Z10" s="4"/>
     </row>
     <row r="11" spans="1:26" ht="9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="137"/>
-      <c r="B11" s="137"/>
-      <c r="C11" s="137"/>
-      <c r="D11" s="137"/>
-      <c r="E11" s="137"/>
-      <c r="F11" s="137"/>
-      <c r="G11" s="137"/>
+      <c r="A11" s="136"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="136"/>
+      <c r="D11" s="136"/>
+      <c r="E11" s="136"/>
+      <c r="F11" s="136"/>
+      <c r="G11" s="136"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -12762,9 +12762,9 @@
       <c r="B12" s="135" t="s">
         <v>318</v>
       </c>
-      <c r="C12" s="137"/>
-      <c r="D12" s="137"/>
-      <c r="E12" s="137"/>
+      <c r="C12" s="136"/>
+      <c r="D12" s="136"/>
+      <c r="E12" s="136"/>
       <c r="F12" s="135" t="s">
         <v>256</v>
       </c>
@@ -12794,13 +12794,13 @@
       <c r="A13" s="47" t="s">
         <v>320</v>
       </c>
-      <c r="B13" s="136" t="s">
+      <c r="B13" s="137" t="s">
         <v>321</v>
       </c>
-      <c r="C13" s="137"/>
-      <c r="D13" s="137"/>
-      <c r="E13" s="137"/>
-      <c r="F13" s="136"/>
+      <c r="C13" s="136"/>
+      <c r="D13" s="136"/>
+      <c r="E13" s="136"/>
+      <c r="F13" s="137"/>
       <c r="G13" s="47" t="s">
         <v>322</v>
       </c>
@@ -12828,12 +12828,12 @@
       <c r="A14" s="135" t="s">
         <v>323</v>
       </c>
-      <c r="B14" s="139" t="s">
+      <c r="B14" s="140" t="s">
         <v>324</v>
       </c>
-      <c r="C14" s="137"/>
-      <c r="D14" s="137"/>
-      <c r="E14" s="137"/>
+      <c r="C14" s="136"/>
+      <c r="D14" s="136"/>
+      <c r="E14" s="136"/>
       <c r="F14" s="135" t="s">
         <v>325</v>
       </c>
@@ -12861,13 +12861,13 @@
       <c r="Z14" s="4"/>
     </row>
     <row r="15" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="137"/>
-      <c r="B15" s="137"/>
-      <c r="C15" s="137"/>
-      <c r="D15" s="137"/>
-      <c r="E15" s="137"/>
-      <c r="F15" s="137"/>
-      <c r="G15" s="137"/>
+      <c r="A15" s="136"/>
+      <c r="B15" s="136"/>
+      <c r="C15" s="136"/>
+      <c r="D15" s="136"/>
+      <c r="E15" s="136"/>
+      <c r="F15" s="136"/>
+      <c r="G15" s="136"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
@@ -12892,12 +12892,12 @@
       <c r="A16" s="135" t="s">
         <v>327</v>
       </c>
-      <c r="B16" s="139" t="s">
+      <c r="B16" s="140" t="s">
         <v>328</v>
       </c>
-      <c r="C16" s="137"/>
-      <c r="D16" s="137"/>
-      <c r="E16" s="137"/>
+      <c r="C16" s="136"/>
+      <c r="D16" s="136"/>
+      <c r="E16" s="136"/>
       <c r="F16" s="135" t="s">
         <v>329</v>
       </c>
@@ -12925,13 +12925,13 @@
       <c r="Z16" s="4"/>
     </row>
     <row r="17" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="137"/>
-      <c r="B17" s="137"/>
-      <c r="C17" s="137"/>
-      <c r="D17" s="137"/>
-      <c r="E17" s="137"/>
-      <c r="F17" s="137"/>
-      <c r="G17" s="137"/>
+      <c r="A17" s="136"/>
+      <c r="B17" s="136"/>
+      <c r="C17" s="136"/>
+      <c r="D17" s="136"/>
+      <c r="E17" s="136"/>
+      <c r="F17" s="136"/>
+      <c r="G17" s="136"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
@@ -12953,13 +12953,13 @@
       <c r="Z17" s="4"/>
     </row>
     <row r="18" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="137"/>
-      <c r="B18" s="137"/>
-      <c r="C18" s="137"/>
-      <c r="D18" s="137"/>
-      <c r="E18" s="137"/>
-      <c r="F18" s="137"/>
-      <c r="G18" s="137"/>
+      <c r="A18" s="136"/>
+      <c r="B18" s="136"/>
+      <c r="C18" s="136"/>
+      <c r="D18" s="136"/>
+      <c r="E18" s="136"/>
+      <c r="F18" s="136"/>
+      <c r="G18" s="136"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -12981,19 +12981,19 @@
       <c r="Z18" s="4"/>
     </row>
     <row r="19" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="136" t="s">
+      <c r="A19" s="137" t="s">
         <v>331</v>
       </c>
-      <c r="B19" s="140" t="s">
+      <c r="B19" s="144" t="s">
         <v>332</v>
       </c>
-      <c r="C19" s="137"/>
-      <c r="D19" s="137"/>
-      <c r="E19" s="137"/>
-      <c r="F19" s="136" t="s">
+      <c r="C19" s="136"/>
+      <c r="D19" s="136"/>
+      <c r="E19" s="136"/>
+      <c r="F19" s="137" t="s">
         <v>333</v>
       </c>
-      <c r="G19" s="136" t="s">
+      <c r="G19" s="137" t="s">
         <v>334</v>
       </c>
       <c r="I19" s="4"/>
@@ -13016,13 +13016,13 @@
       <c r="Z19" s="4"/>
     </row>
     <row r="20" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="137"/>
-      <c r="B20" s="137"/>
-      <c r="C20" s="137"/>
-      <c r="D20" s="137"/>
-      <c r="E20" s="137"/>
-      <c r="F20" s="137"/>
-      <c r="G20" s="137"/>
+      <c r="A20" s="136"/>
+      <c r="B20" s="136"/>
+      <c r="C20" s="136"/>
+      <c r="D20" s="136"/>
+      <c r="E20" s="136"/>
+      <c r="F20" s="136"/>
+      <c r="G20" s="136"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
@@ -13047,12 +13047,12 @@
       <c r="A21" s="47" t="s">
         <v>335</v>
       </c>
-      <c r="B21" s="136" t="s">
+      <c r="B21" s="137" t="s">
         <v>336</v>
       </c>
-      <c r="C21" s="137"/>
-      <c r="D21" s="137"/>
-      <c r="E21" s="137"/>
+      <c r="C21" s="136"/>
+      <c r="D21" s="136"/>
+      <c r="E21" s="136"/>
       <c r="F21" s="47" t="s">
         <v>337</v>
       </c>
@@ -13083,12 +13083,12 @@
       <c r="A22" s="47" t="s">
         <v>342</v>
       </c>
-      <c r="B22" s="136" t="s">
+      <c r="B22" s="137" t="s">
         <v>339</v>
       </c>
-      <c r="C22" s="136"/>
-      <c r="D22" s="136"/>
-      <c r="E22" s="136"/>
+      <c r="C22" s="137"/>
+      <c r="D22" s="137"/>
+      <c r="E22" s="137"/>
       <c r="F22" s="47" t="s">
         <v>340</v>
       </c>
@@ -13155,12 +13155,12 @@
       <c r="A24" s="47" t="s">
         <v>348</v>
       </c>
-      <c r="B24" s="136" t="s">
+      <c r="B24" s="137" t="s">
         <v>346</v>
       </c>
-      <c r="C24" s="136"/>
-      <c r="D24" s="136"/>
-      <c r="E24" s="136"/>
+      <c r="C24" s="137"/>
+      <c r="D24" s="137"/>
+      <c r="E24" s="137"/>
       <c r="F24" s="47" t="s">
         <v>340</v>
       </c>
@@ -13227,12 +13227,12 @@
       <c r="A26" s="47" t="s">
         <v>355</v>
       </c>
-      <c r="B26" s="136" t="s">
+      <c r="B26" s="137" t="s">
         <v>352</v>
       </c>
-      <c r="C26" s="136"/>
-      <c r="D26" s="136"/>
-      <c r="E26" s="136"/>
+      <c r="C26" s="137"/>
+      <c r="D26" s="137"/>
+      <c r="E26" s="137"/>
       <c r="F26" s="47" t="s">
         <v>353</v>
       </c>
@@ -13299,12 +13299,12 @@
       <c r="A28" s="47" t="s">
         <v>361</v>
       </c>
-      <c r="B28" s="136" t="s">
+      <c r="B28" s="137" t="s">
         <v>359</v>
       </c>
-      <c r="C28" s="136"/>
-      <c r="D28" s="136"/>
-      <c r="E28" s="136"/>
+      <c r="C28" s="137"/>
+      <c r="D28" s="137"/>
+      <c r="E28" s="137"/>
       <c r="F28" s="47" t="s">
         <v>353</v>
       </c>
@@ -13371,12 +13371,12 @@
       <c r="A30" s="47" t="s">
         <v>368</v>
       </c>
-      <c r="B30" s="136" t="s">
+      <c r="B30" s="137" t="s">
         <v>366</v>
       </c>
-      <c r="C30" s="136"/>
-      <c r="D30" s="136"/>
-      <c r="E30" s="136"/>
+      <c r="C30" s="137"/>
+      <c r="D30" s="137"/>
+      <c r="E30" s="137"/>
       <c r="F30" s="47" t="s">
         <v>363</v>
       </c>
@@ -13443,12 +13443,12 @@
       <c r="A32" s="47" t="s">
         <v>374</v>
       </c>
-      <c r="B32" s="136" t="s">
+      <c r="B32" s="137" t="s">
         <v>372</v>
       </c>
-      <c r="C32" s="136"/>
-      <c r="D32" s="136"/>
-      <c r="E32" s="136"/>
+      <c r="C32" s="137"/>
+      <c r="D32" s="137"/>
+      <c r="E32" s="137"/>
       <c r="F32" s="47" t="s">
         <v>363</v>
       </c>
@@ -13515,12 +13515,12 @@
       <c r="A34" s="47" t="s">
         <v>382</v>
       </c>
-      <c r="B34" s="136" t="s">
+      <c r="B34" s="137" t="s">
         <v>379</v>
       </c>
-      <c r="C34" s="136"/>
-      <c r="D34" s="136"/>
-      <c r="E34" s="136"/>
+      <c r="C34" s="137"/>
+      <c r="D34" s="137"/>
+      <c r="E34" s="137"/>
       <c r="F34" s="47" t="s">
         <v>380</v>
       </c>
@@ -13587,12 +13587,12 @@
       <c r="A36" s="47" t="s">
         <v>388</v>
       </c>
-      <c r="B36" s="136" t="s">
+      <c r="B36" s="137" t="s">
         <v>386</v>
       </c>
-      <c r="C36" s="136"/>
-      <c r="D36" s="136"/>
-      <c r="E36" s="136"/>
+      <c r="C36" s="137"/>
+      <c r="D36" s="137"/>
+      <c r="E36" s="137"/>
       <c r="F36" s="47" t="s">
         <v>337</v>
       </c>
@@ -13659,12 +13659,12 @@
       <c r="A38" s="47" t="s">
         <v>394</v>
       </c>
-      <c r="B38" s="136" t="s">
+      <c r="B38" s="137" t="s">
         <v>392</v>
       </c>
-      <c r="C38" s="136"/>
-      <c r="D38" s="136"/>
-      <c r="E38" s="136"/>
+      <c r="C38" s="137"/>
+      <c r="D38" s="137"/>
+      <c r="E38" s="137"/>
       <c r="F38" s="47" t="s">
         <v>337</v>
       </c>
@@ -13729,14 +13729,14 @@
     </row>
     <row r="40" spans="1:26" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="47" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
-      <c r="B40" s="137" t="s">
+      <c r="B40" s="136" t="s">
         <v>399</v>
       </c>
-      <c r="C40" s="137"/>
-      <c r="D40" s="137"/>
-      <c r="E40" s="137"/>
+      <c r="C40" s="136"/>
+      <c r="D40" s="136"/>
+      <c r="E40" s="136"/>
       <c r="F40" s="47" t="s">
         <v>396</v>
       </c>
@@ -21573,21 +21573,21 @@
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="F4:F7"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B14:E15"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B8:E11"/>
-    <mergeCell ref="F8:F11"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="B16:E18"/>
-    <mergeCell ref="B19:E20"/>
-    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:E35"/>
     <mergeCell ref="B38:E38"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B40:E40"/>
@@ -21604,21 +21604,21 @@
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B4:E7"/>
     <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B8:E11"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="B16:E18"/>
+    <mergeCell ref="B19:E20"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="F4:F7"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B14:E15"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="A14:A15"/>
   </mergeCells>
   <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -21652,36 +21652,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:111" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="147"/>
-      <c r="B1" s="121"/>
-      <c r="C1" s="146" t="s">
+      <c r="A1" s="161"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="160" t="s">
         <v>401</v>
       </c>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="157" t="s">
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="118"/>
+      <c r="J1" s="162" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1" s="151"/>
+      <c r="L1" s="151"/>
+      <c r="M1" s="151"/>
+      <c r="N1" s="151"/>
+      <c r="O1" s="151"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="151"/>
+      <c r="R1" s="151"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="149"/>
+      <c r="U1" s="146" t="s">
         <v>402</v>
       </c>
-      <c r="K1" s="158"/>
-      <c r="L1" s="158"/>
-      <c r="M1" s="158"/>
-      <c r="N1" s="158"/>
-      <c r="O1" s="158"/>
-      <c r="P1" s="158"/>
-      <c r="Q1" s="158"/>
-      <c r="R1" s="158"/>
-      <c r="S1" s="158"/>
-      <c r="T1" s="159"/>
-      <c r="U1" s="160" t="s">
-        <v>403</v>
-      </c>
-      <c r="V1" s="149"/>
-      <c r="W1" s="149"/>
-      <c r="X1" s="149"/>
+      <c r="V1" s="147"/>
+      <c r="W1" s="147"/>
+      <c r="X1" s="147"/>
       <c r="Y1" s="15"/>
       <c r="Z1" s="15"/>
       <c r="AA1" s="15"/>
@@ -21771,59 +21771,59 @@
       <c r="DG1" s="16"/>
     </row>
     <row r="2" spans="1:111" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121"/>
-      <c r="B2" s="121"/>
+      <c r="A2" s="118"/>
+      <c r="B2" s="118"/>
       <c r="C2" s="17" t="s">
+        <v>403</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>404</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="E2" s="17" t="s">
         <v>405</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="F2" s="17" t="s">
         <v>406</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="G2" s="17" t="s">
         <v>407</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="H2" s="17" t="s">
         <v>408</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>409</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="J2" s="148" t="s">
         <v>410</v>
       </c>
-      <c r="J2" s="161" t="s">
+      <c r="K2" s="151"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="148" t="s">
         <v>411</v>
       </c>
-      <c r="K2" s="158"/>
-      <c r="L2" s="159"/>
-      <c r="M2" s="161" t="s">
+      <c r="N2" s="149"/>
+      <c r="O2" s="148" t="s">
         <v>412</v>
       </c>
-      <c r="N2" s="159"/>
-      <c r="O2" s="161" t="s">
+      <c r="P2" s="151"/>
+      <c r="Q2" s="149"/>
+      <c r="R2" s="148" t="s">
         <v>413</v>
       </c>
-      <c r="P2" s="158"/>
-      <c r="Q2" s="159"/>
-      <c r="R2" s="161" t="s">
+      <c r="S2" s="151"/>
+      <c r="T2" s="149"/>
+      <c r="U2" s="19" t="s">
         <v>414</v>
       </c>
-      <c r="S2" s="158"/>
-      <c r="T2" s="159"/>
-      <c r="U2" s="19" t="s">
+      <c r="V2" s="20" t="s">
         <v>415</v>
       </c>
-      <c r="V2" s="20" t="s">
+      <c r="W2" s="20" t="s">
         <v>416</v>
       </c>
-      <c r="W2" s="20" t="s">
+      <c r="X2" s="20" t="s">
         <v>417</v>
-      </c>
-      <c r="X2" s="20" t="s">
-        <v>418</v>
       </c>
       <c r="Y2" s="21"/>
       <c r="Z2" s="15"/>
@@ -21915,13 +21915,13 @@
     </row>
     <row r="3" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="163" t="s">
+        <v>418</v>
+      </c>
+      <c r="B3" s="23" t="s">
         <v>419</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="C3" s="24" t="s">
         <v>420</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>421</v>
       </c>
       <c r="D3" s="25"/>
       <c r="E3" s="25"/>
@@ -21929,21 +21929,21 @@
       <c r="G3" s="25"/>
       <c r="H3" s="25"/>
       <c r="I3" s="25"/>
-      <c r="J3" s="148" t="s">
-        <v>421</v>
+      <c r="J3" s="152" t="s">
+        <v>420</v>
       </c>
-      <c r="K3" s="149"/>
-      <c r="L3" s="150"/>
-      <c r="M3" s="154"/>
-      <c r="N3" s="150"/>
-      <c r="O3" s="148" t="s">
-        <v>421</v>
+      <c r="K3" s="147"/>
+      <c r="L3" s="153"/>
+      <c r="M3" s="156"/>
+      <c r="N3" s="153"/>
+      <c r="O3" s="152" t="s">
+        <v>420</v>
       </c>
-      <c r="P3" s="149"/>
-      <c r="Q3" s="150"/>
-      <c r="R3" s="162"/>
-      <c r="S3" s="149"/>
-      <c r="T3" s="149"/>
+      <c r="P3" s="147"/>
+      <c r="Q3" s="153"/>
+      <c r="R3" s="150"/>
+      <c r="S3" s="147"/>
+      <c r="T3" s="147"/>
       <c r="U3" s="26"/>
       <c r="V3" s="26"/>
       <c r="W3" s="26"/>
@@ -22039,32 +22039,32 @@
     <row r="4" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="164"/>
       <c r="B4" s="27" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
-      <c r="J4" s="152"/>
-      <c r="K4" s="142"/>
-      <c r="L4" s="134"/>
-      <c r="M4" s="151" t="s">
-        <v>421</v>
+      <c r="J4" s="155"/>
+      <c r="K4" s="139"/>
+      <c r="L4" s="124"/>
+      <c r="M4" s="159" t="s">
+        <v>420</v>
       </c>
-      <c r="N4" s="134"/>
-      <c r="O4" s="152"/>
-      <c r="P4" s="142"/>
-      <c r="Q4" s="134"/>
-      <c r="R4" s="156"/>
-      <c r="S4" s="142"/>
-      <c r="T4" s="142"/>
+      <c r="N4" s="124"/>
+      <c r="O4" s="155"/>
+      <c r="P4" s="139"/>
+      <c r="Q4" s="124"/>
+      <c r="R4" s="158"/>
+      <c r="S4" s="139"/>
+      <c r="T4" s="139"/>
       <c r="U4" s="26"/>
       <c r="V4" s="26"/>
       <c r="W4" s="26"/>
@@ -22160,30 +22160,30 @@
     <row r="5" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="164"/>
       <c r="B5" s="27" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C5" s="28"/>
       <c r="D5" s="16"/>
       <c r="E5" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F5" s="29"/>
       <c r="G5" s="29"/>
       <c r="H5" s="29"/>
       <c r="I5" s="29"/>
-      <c r="J5" s="152"/>
-      <c r="K5" s="142"/>
-      <c r="L5" s="134"/>
-      <c r="M5" s="151" t="s">
-        <v>421</v>
+      <c r="J5" s="155"/>
+      <c r="K5" s="139"/>
+      <c r="L5" s="124"/>
+      <c r="M5" s="159" t="s">
+        <v>420</v>
       </c>
-      <c r="N5" s="134"/>
-      <c r="O5" s="152"/>
-      <c r="P5" s="142"/>
-      <c r="Q5" s="134"/>
-      <c r="R5" s="156"/>
-      <c r="S5" s="142"/>
-      <c r="T5" s="142"/>
+      <c r="N5" s="124"/>
+      <c r="O5" s="155"/>
+      <c r="P5" s="139"/>
+      <c r="Q5" s="124"/>
+      <c r="R5" s="158"/>
+      <c r="S5" s="139"/>
+      <c r="T5" s="139"/>
       <c r="U5" s="26"/>
       <c r="V5" s="26"/>
       <c r="W5" s="26"/>
@@ -22279,30 +22279,30 @@
     <row r="6" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="164"/>
       <c r="B6" s="27" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C6" s="28"/>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
       <c r="F6" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G6" s="29"/>
       <c r="H6" s="29"/>
       <c r="I6" s="29"/>
-      <c r="J6" s="152"/>
-      <c r="K6" s="142"/>
-      <c r="L6" s="134"/>
-      <c r="M6" s="151" t="s">
-        <v>421</v>
+      <c r="J6" s="155"/>
+      <c r="K6" s="139"/>
+      <c r="L6" s="124"/>
+      <c r="M6" s="159" t="s">
+        <v>420</v>
       </c>
-      <c r="N6" s="134"/>
-      <c r="O6" s="152"/>
-      <c r="P6" s="142"/>
-      <c r="Q6" s="134"/>
-      <c r="R6" s="156"/>
-      <c r="S6" s="142"/>
-      <c r="T6" s="142"/>
+      <c r="N6" s="124"/>
+      <c r="O6" s="155"/>
+      <c r="P6" s="139"/>
+      <c r="Q6" s="124"/>
+      <c r="R6" s="158"/>
+      <c r="S6" s="139"/>
+      <c r="T6" s="139"/>
       <c r="U6" s="26"/>
       <c r="V6" s="26"/>
       <c r="W6" s="26"/>
@@ -22398,30 +22398,30 @@
     <row r="7" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="164"/>
       <c r="B7" s="27" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C7" s="28"/>
       <c r="D7" s="16"/>
       <c r="E7" s="11"/>
       <c r="F7" s="29"/>
       <c r="G7" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H7" s="29"/>
       <c r="I7" s="29"/>
-      <c r="J7" s="152"/>
-      <c r="K7" s="142"/>
-      <c r="L7" s="134"/>
-      <c r="M7" s="151" t="s">
-        <v>421</v>
+      <c r="J7" s="155"/>
+      <c r="K7" s="139"/>
+      <c r="L7" s="124"/>
+      <c r="M7" s="159" t="s">
+        <v>420</v>
       </c>
-      <c r="N7" s="134"/>
-      <c r="O7" s="152"/>
-      <c r="P7" s="142"/>
-      <c r="Q7" s="134"/>
-      <c r="R7" s="156"/>
-      <c r="S7" s="142"/>
-      <c r="T7" s="142"/>
+      <c r="N7" s="124"/>
+      <c r="O7" s="155"/>
+      <c r="P7" s="139"/>
+      <c r="Q7" s="124"/>
+      <c r="R7" s="158"/>
+      <c r="S7" s="139"/>
+      <c r="T7" s="139"/>
       <c r="U7" s="26"/>
       <c r="V7" s="26"/>
       <c r="W7" s="26"/>
@@ -22517,7 +22517,7 @@
     <row r="8" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="164"/>
       <c r="B8" s="27" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C8" s="28"/>
       <c r="D8" s="11"/>
@@ -22525,22 +22525,22 @@
       <c r="F8" s="29"/>
       <c r="G8" s="29"/>
       <c r="H8" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I8" s="29"/>
-      <c r="J8" s="152"/>
-      <c r="K8" s="142"/>
-      <c r="L8" s="134"/>
-      <c r="M8" s="151" t="s">
-        <v>421</v>
+      <c r="J8" s="155"/>
+      <c r="K8" s="139"/>
+      <c r="L8" s="124"/>
+      <c r="M8" s="159" t="s">
+        <v>420</v>
       </c>
-      <c r="N8" s="134"/>
+      <c r="N8" s="124"/>
       <c r="O8" s="165"/>
-      <c r="P8" s="142"/>
-      <c r="Q8" s="134"/>
-      <c r="R8" s="155"/>
-      <c r="S8" s="142"/>
-      <c r="T8" s="142"/>
+      <c r="P8" s="139"/>
+      <c r="Q8" s="124"/>
+      <c r="R8" s="157"/>
+      <c r="S8" s="139"/>
+      <c r="T8" s="139"/>
       <c r="U8" s="26"/>
       <c r="V8" s="26"/>
       <c r="W8" s="26"/>
@@ -22636,7 +22636,7 @@
     <row r="9" spans="1:111" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="164"/>
       <c r="B9" s="27" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C9" s="28"/>
       <c r="D9" s="11"/>
@@ -22645,21 +22645,21 @@
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
       <c r="I9" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
-      <c r="J9" s="152"/>
-      <c r="K9" s="142"/>
-      <c r="L9" s="134"/>
-      <c r="M9" s="151"/>
-      <c r="N9" s="134"/>
-      <c r="O9" s="151"/>
-      <c r="P9" s="142"/>
-      <c r="Q9" s="134"/>
-      <c r="R9" s="153" t="s">
-        <v>421</v>
+      <c r="J9" s="155"/>
+      <c r="K9" s="139"/>
+      <c r="L9" s="124"/>
+      <c r="M9" s="159"/>
+      <c r="N9" s="124"/>
+      <c r="O9" s="159"/>
+      <c r="P9" s="139"/>
+      <c r="Q9" s="124"/>
+      <c r="R9" s="154" t="s">
+        <v>420</v>
       </c>
-      <c r="S9" s="142"/>
-      <c r="T9" s="142"/>
+      <c r="S9" s="139"/>
+      <c r="T9" s="139"/>
       <c r="U9" s="26"/>
       <c r="V9" s="26"/>
       <c r="W9" s="26"/>
@@ -22763,7 +22763,7 @@
       <c r="H10" s="31"/>
       <c r="I10" s="31"/>
       <c r="J10" s="32" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K10" s="33"/>
       <c r="L10" s="33"/>
@@ -28575,7 +28575,7 @@
       <c r="BC61" s="31"/>
       <c r="BD61" s="31"/>
       <c r="BE61" s="31" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BF61" s="31"/>
       <c r="BG61" s="31"/>
@@ -28811,7 +28811,7 @@
       <c r="BK63" s="34"/>
       <c r="BL63" s="34"/>
       <c r="BM63" s="31" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BN63" s="34"/>
       <c r="BO63" s="34"/>
@@ -28924,7 +28924,7 @@
       <c r="BI64" s="31"/>
       <c r="BJ64" s="34"/>
       <c r="BK64" s="31" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BL64" s="34"/>
       <c r="BM64" s="34"/>
@@ -29156,7 +29156,7 @@
       <c r="BM66" s="34"/>
       <c r="BN66" s="34"/>
       <c r="BO66" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BP66" s="34"/>
       <c r="BQ66" s="34"/>
@@ -29384,7 +29384,7 @@
       <c r="BM68" s="34"/>
       <c r="BN68" s="34"/>
       <c r="BO68" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BP68" s="34"/>
       <c r="BQ68" s="34"/>
@@ -29496,7 +29496,7 @@
       <c r="BJ69" s="34"/>
       <c r="BK69" s="34"/>
       <c r="BL69" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BM69" s="34"/>
       <c r="BN69" s="34"/>
@@ -29730,7 +29730,7 @@
       <c r="BP71" s="34"/>
       <c r="BQ71" s="34"/>
       <c r="BR71" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BS71" s="35"/>
       <c r="BT71" s="12"/>
@@ -29848,7 +29848,7 @@
       <c r="BS72" s="12"/>
       <c r="BT72" s="35"/>
       <c r="BU72" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BV72" s="12"/>
       <c r="BW72" s="12"/>
@@ -30076,7 +30076,7 @@
       <c r="BS74" s="12"/>
       <c r="BT74" s="12"/>
       <c r="BU74" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BV74" s="35"/>
       <c r="BW74" s="12"/>
@@ -30191,7 +30191,7 @@
       <c r="BS75" s="12"/>
       <c r="BT75" s="12"/>
       <c r="BU75" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BV75" s="34"/>
       <c r="BW75" s="35"/>
@@ -30304,13 +30304,13 @@
       <c r="BQ76" s="34"/>
       <c r="BR76" s="12"/>
       <c r="BS76" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BT76" s="12"/>
       <c r="BU76" s="12"/>
       <c r="BV76" s="12"/>
       <c r="BW76" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BX76" s="35"/>
       <c r="BY76" s="12"/>
@@ -30540,7 +30540,7 @@
       <c r="BW78" s="12"/>
       <c r="BX78" s="12"/>
       <c r="BY78" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BZ78" s="35"/>
       <c r="CA78" s="12"/>
@@ -30658,7 +30658,7 @@
       <c r="BZ79" s="12"/>
       <c r="CA79" s="35"/>
       <c r="CB79" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CC79" s="12"/>
       <c r="CD79" s="12"/>
@@ -30886,7 +30886,7 @@
       <c r="BZ81" s="12"/>
       <c r="CA81" s="12"/>
       <c r="CB81" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CC81" s="35"/>
       <c r="CD81" s="12"/>
@@ -30999,7 +30999,7 @@
       <c r="BX82" s="12"/>
       <c r="BY82" s="12"/>
       <c r="BZ82" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CA82" s="12"/>
       <c r="CB82" s="12"/>
@@ -31235,7 +31235,7 @@
       <c r="CF84" s="35"/>
       <c r="CG84" s="12"/>
       <c r="CH84" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CI84" s="12"/>
       <c r="CJ84" s="12"/>
@@ -31348,7 +31348,7 @@
       <c r="CD85" s="12"/>
       <c r="CE85" s="12"/>
       <c r="CF85" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CG85" s="35"/>
       <c r="CH85" s="12"/>
@@ -31580,7 +31580,7 @@
       <c r="CH87" s="12"/>
       <c r="CI87" s="35"/>
       <c r="CJ87" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CK87" s="12"/>
       <c r="CL87" s="12"/>
@@ -31808,7 +31808,7 @@
       <c r="CH89" s="12"/>
       <c r="CI89" s="12"/>
       <c r="CJ89" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CK89" s="35"/>
       <c r="CL89" s="12"/>
@@ -31923,7 +31923,7 @@
       <c r="CH90" s="12"/>
       <c r="CI90" s="12"/>
       <c r="CJ90" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CK90" s="12"/>
       <c r="CL90" s="35"/>
@@ -32035,14 +32035,14 @@
       <c r="CE91" s="12"/>
       <c r="CF91" s="12"/>
       <c r="CG91" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CH91" s="12"/>
       <c r="CI91" s="12"/>
       <c r="CJ91" s="12"/>
       <c r="CK91" s="12"/>
       <c r="CL91" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CM91" s="35"/>
       <c r="CN91" s="12"/>
@@ -32160,7 +32160,7 @@
       <c r="CM92" s="12"/>
       <c r="CN92" s="35"/>
       <c r="CO92" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CP92" s="12"/>
       <c r="CQ92" s="12"/>
@@ -32387,7 +32387,7 @@
       <c r="CL94" s="12"/>
       <c r="CM94" s="12"/>
       <c r="CN94" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CO94" s="12"/>
       <c r="CP94" s="35"/>
@@ -32506,7 +32506,7 @@
       <c r="CP95" s="12"/>
       <c r="CQ95" s="35"/>
       <c r="CR95" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CS95" s="12"/>
       <c r="CT95" s="12"/>
@@ -32847,7 +32847,7 @@
       <c r="CP98" s="12"/>
       <c r="CQ98" s="12"/>
       <c r="CR98" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CS98" s="34"/>
       <c r="CT98" s="35"/>
@@ -32964,7 +32964,7 @@
       <c r="CR99" s="12"/>
       <c r="CS99" s="12"/>
       <c r="CT99" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CU99" s="35"/>
       <c r="CV99" s="34"/>
@@ -33077,7 +33077,7 @@
       <c r="CP100" s="12"/>
       <c r="CQ100" s="12"/>
       <c r="CR100" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CS100" s="12"/>
       <c r="CT100" s="12"/>
@@ -33310,7 +33310,7 @@
       <c r="CU102" s="12"/>
       <c r="CV102" s="12"/>
       <c r="CW102" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CX102" s="35"/>
       <c r="CY102" s="12"/>
@@ -33428,7 +33428,7 @@
       <c r="CX103" s="12"/>
       <c r="CY103" s="35"/>
       <c r="CZ103" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="DA103" s="12"/>
       <c r="DB103" s="12"/>
@@ -33656,7 +33656,7 @@
       <c r="CX105" s="12"/>
       <c r="CY105" s="12"/>
       <c r="CZ105" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="DA105" s="35"/>
       <c r="DB105" s="12"/>
@@ -33769,7 +33769,7 @@
       <c r="CV106" s="12"/>
       <c r="CW106" s="12"/>
       <c r="CX106" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CY106" s="12"/>
       <c r="CZ106" s="12"/>
@@ -33836,7 +33836,7 @@
       <c r="AZ107" s="31"/>
       <c r="BA107" s="31"/>
       <c r="BB107" s="31" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BC107" s="31"/>
       <c r="BD107" s="31"/>
@@ -33853,7 +33853,7 @@
       <c r="BO107" s="34"/>
       <c r="BP107" s="34"/>
       <c r="BQ107" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BR107" s="12"/>
       <c r="BS107" s="12"/>
@@ -33862,7 +33862,7 @@
       <c r="BV107" s="12"/>
       <c r="BW107" s="12"/>
       <c r="BX107" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BY107" s="12"/>
       <c r="BZ107" s="12"/>
@@ -33870,7 +33870,7 @@
       <c r="CB107" s="12"/>
       <c r="CC107" s="12"/>
       <c r="CD107" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CE107" s="12"/>
       <c r="CF107" s="12"/>
@@ -33957,7 +33957,7 @@
       <c r="AZ108" s="31"/>
       <c r="BA108" s="31"/>
       <c r="BB108" s="31" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BC108" s="31"/>
       <c r="BD108" s="31"/>
@@ -33974,7 +33974,7 @@
       <c r="BO108" s="34"/>
       <c r="BP108" s="34"/>
       <c r="BQ108" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BR108" s="12"/>
       <c r="BS108" s="12"/>
@@ -33983,7 +33983,7 @@
       <c r="BV108" s="12"/>
       <c r="BW108" s="12"/>
       <c r="BX108" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BY108" s="12"/>
       <c r="BZ108" s="12"/>
@@ -33991,7 +33991,7 @@
       <c r="CB108" s="12"/>
       <c r="CC108" s="12"/>
       <c r="CD108" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CE108" s="12"/>
       <c r="CF108" s="12"/>
@@ -34084,7 +34084,7 @@
       <c r="BF109" s="31"/>
       <c r="BG109" s="31"/>
       <c r="BH109" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BI109" s="31"/>
       <c r="BJ109" s="34"/>
@@ -34117,12 +34117,12 @@
       <c r="CK109" s="12"/>
       <c r="CL109" s="12"/>
       <c r="CM109" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CN109" s="12"/>
       <c r="CO109" s="12"/>
       <c r="CP109" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CQ109" s="12"/>
       <c r="CR109" s="12"/>
@@ -34136,7 +34136,7 @@
       <c r="CZ109" s="12"/>
       <c r="DA109" s="12"/>
       <c r="DB109" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="DC109" s="12"/>
       <c r="DD109" s="34"/>
@@ -34205,7 +34205,7 @@
       <c r="BF110" s="31"/>
       <c r="BG110" s="31"/>
       <c r="BH110" s="34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="BI110" s="31"/>
       <c r="BJ110" s="34"/>
@@ -34238,12 +34238,12 @@
       <c r="CK110" s="12"/>
       <c r="CL110" s="12"/>
       <c r="CM110" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CN110" s="12"/>
       <c r="CO110" s="12"/>
       <c r="CP110" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="CQ110" s="12"/>
       <c r="CR110" s="12"/>
@@ -34257,7 +34257,7 @@
       <c r="CZ110" s="12"/>
       <c r="DA110" s="12"/>
       <c r="DB110" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="DC110" s="12"/>
       <c r="DD110" s="12"/>
@@ -56867,13 +56867,20 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="R3:T3"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="O6:Q6"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="J1:T1"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="A3:A9"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="O8:Q8"/>
     <mergeCell ref="R9:T9"/>
     <mergeCell ref="J8:L8"/>
     <mergeCell ref="O7:Q7"/>
@@ -56890,20 +56897,13 @@
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="R5:T5"/>
     <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="O6:Q6"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="J1:T1"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="A3:A9"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="O8:Q8"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="R3:T3"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="R2:T2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>